<commit_message>
feat(repeat): aqueous-only tubes; round 2 adds B2 B3 B4 BIN6 (aq), BIN8, I4 (aq)
'TUBE:aq' on the --round command line: the entry sheet lists only that tube's aqueous
vials (so repeat_results patches only those; the organic phase stays campaign 1's), the
prep book labels it '(aq only)'. Round 2 is now A1-A5 BIN1 F5 I2 B2:aq B3:aq B4:aq BIN6:aq
BIN8 I4:aq (14 tubes, 46 vials); TENTATIVE gains B2 B3 B4 F-bin I-bin I4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat2_entry.xlsx
+++ b/out/repeat2_entry.xlsx
@@ -279,24 +279,34 @@
         <t>Campaign 1: 1.4736 %</t>
       </text>
     </comment>
-    <comment ref="M33" authorId="0" shapeId="0">
+    <comment ref="M39" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.8273 %</t>
       </text>
     </comment>
-    <comment ref="M34" authorId="0" shapeId="0">
+    <comment ref="M40" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.7719 %</t>
       </text>
     </comment>
-    <comment ref="M39" authorId="0" shapeId="0">
+    <comment ref="M47" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.9451 %</t>
       </text>
     </comment>
-    <comment ref="M40" authorId="0" shapeId="0">
+    <comment ref="M48" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.908 %</t>
+      </text>
+    </comment>
+    <comment ref="M53" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 1.6475 %</t>
+      </text>
+    </comment>
+    <comment ref="M54" authorId="0" shapeId="0">
+      <text>
+        <t>Campaign 1: 1.6484 %</t>
       </text>
     </comment>
   </commentList>
@@ -592,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2170,22 +2180,22 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>F5-T1</t>
+          <t>B2-B1</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E33" s="12" t="n"/>
@@ -2210,11 +2220,11 @@
         <f>IF(AND(ISNUMBER(J33),ISNUMBER(K33)),IF(J33&gt;0,(J33+K33)/J33,""),"")</f>
         <v/>
       </c>
-      <c r="M33" s="13" t="n"/>
-      <c r="N33" s="13" t="n"/>
+      <c r="M33" s="20" t="n"/>
+      <c r="N33" s="20" t="n"/>
       <c r="O33" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P33" s="13" t="n"/>
@@ -2222,22 +2232,22 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>F5-T2</t>
+          <t>B2-B2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E34" s="16" t="n"/>
@@ -2262,76 +2272,76 @@
         <f>IF(AND(ISNUMBER(J34),ISNUMBER(K34)),IF(J34&gt;0,(J34+K34)/J34,""),"")</f>
         <v/>
       </c>
-      <c r="M34" s="17" t="n"/>
-      <c r="N34" s="17" t="n"/>
+      <c r="M34" s="5" t="n"/>
+      <c r="N34" s="5" t="n"/>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P34" s="17" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>F5-B1</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>B3-B1</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="3">
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="11">
         <f>1000-F35</f>
         <v/>
       </c>
-      <c r="I35" s="16" t="n"/>
-      <c r="J35" s="18">
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="14">
         <f>IF(AND(ISNUMBER(E35),ISNUMBER(G35)),G35-E35,"")</f>
         <v/>
       </c>
-      <c r="K35" s="18">
+      <c r="K35" s="14">
         <f>IF(AND(ISNUMBER(G35),ISNUMBER(I35)),I35-G35,"")</f>
         <v/>
       </c>
-      <c r="L35" s="19">
+      <c r="L35" s="15">
         <f>IF(AND(ISNUMBER(J35),ISNUMBER(K35)),IF(J35&gt;0,(J35+K35)/J35,""),"")</f>
         <v/>
       </c>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="5" t="n"/>
-      <c r="O35" s="3" t="inlineStr">
+      <c r="M35" s="20" t="n"/>
+      <c r="N35" s="20" t="n"/>
+      <c r="O35" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P35" s="17" t="n"/>
+      <c r="P35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>F5-B2</t>
+          <t>B3-B2</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2378,17 +2388,17 @@
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>I2-T1</t>
+          <t>B4-B1</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
@@ -2430,17 +2440,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>I2-T2</t>
+          <t>B4-B2</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2480,71 +2490,71 @@
       <c r="P38" s="17" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>I2-B1</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>F5-T1</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>organic</t>
         </is>
       </c>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="3">
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="11">
         <f>1000-F39</f>
         <v/>
       </c>
-      <c r="I39" s="16" t="n"/>
-      <c r="J39" s="18">
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="14">
         <f>IF(AND(ISNUMBER(E39),ISNUMBER(G39)),G39-E39,"")</f>
         <v/>
       </c>
-      <c r="K39" s="18">
+      <c r="K39" s="14">
         <f>IF(AND(ISNUMBER(G39),ISNUMBER(I39)),I39-G39,"")</f>
         <v/>
       </c>
-      <c r="L39" s="19">
+      <c r="L39" s="15">
         <f>IF(AND(ISNUMBER(J39),ISNUMBER(K39)),IF(J39&gt;0,(J39+K39)/J39,""),"")</f>
         <v/>
       </c>
-      <c r="M39" s="17" t="n"/>
-      <c r="N39" s="17" t="n"/>
-      <c r="O39" s="3" t="inlineStr">
+      <c r="M39" s="13" t="n"/>
+      <c r="N39" s="13" t="n"/>
+      <c r="O39" s="11" t="inlineStr">
         <is>
           <t>fresh: type the new KF</t>
         </is>
       </c>
-      <c r="P39" s="17" t="n"/>
+      <c r="P39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>I2-B2</t>
+          <t>F5-T2</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -2583,14 +2593,742 @@
       </c>
       <c r="P40" s="17" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>F5-B1</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="n"/>
+      <c r="F41" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G41" s="16" t="n"/>
+      <c r="H41" s="3">
+        <f>1000-F41</f>
+        <v/>
+      </c>
+      <c r="I41" s="16" t="n"/>
+      <c r="J41" s="18">
+        <f>IF(AND(ISNUMBER(E41),ISNUMBER(G41)),G41-E41,"")</f>
+        <v/>
+      </c>
+      <c r="K41" s="18">
+        <f>IF(AND(ISNUMBER(G41),ISNUMBER(I41)),I41-G41,"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="19">
+        <f>IF(AND(ISNUMBER(J41),ISNUMBER(K41)),IF(J41&gt;0,(J41+K41)/J41,""),"")</f>
+        <v/>
+      </c>
+      <c r="M41" s="5" t="n"/>
+      <c r="N41" s="5" t="n"/>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P41" s="17" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>F5-B2</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="n"/>
+      <c r="F42" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G42" s="16" t="n"/>
+      <c r="H42" s="3">
+        <f>1000-F42</f>
+        <v/>
+      </c>
+      <c r="I42" s="16" t="n"/>
+      <c r="J42" s="18">
+        <f>IF(AND(ISNUMBER(E42),ISNUMBER(G42)),G42-E42,"")</f>
+        <v/>
+      </c>
+      <c r="K42" s="18">
+        <f>IF(AND(ISNUMBER(G42),ISNUMBER(I42)),I42-G42,"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="19">
+        <f>IF(AND(ISNUMBER(J42),ISNUMBER(K42)),IF(J42&gt;0,(J42+K42)/J42,""),"")</f>
+        <v/>
+      </c>
+      <c r="M42" s="5" t="n"/>
+      <c r="N42" s="5" t="n"/>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P42" s="17" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>BIN6</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>BIN6-B1</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="11">
+        <f>1000-F43</f>
+        <v/>
+      </c>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="14">
+        <f>IF(AND(ISNUMBER(E43),ISNUMBER(G43)),G43-E43,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="14">
+        <f>IF(AND(ISNUMBER(G43),ISNUMBER(I43)),I43-G43,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="15">
+        <f>IF(AND(ISNUMBER(J43),ISNUMBER(K43)),IF(J43&gt;0,(J43+K43)/J43,""),"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="20" t="n"/>
+      <c r="N43" s="20" t="n"/>
+      <c r="O43" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>BIN6</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>BIN6-B2</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="n"/>
+      <c r="F44" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G44" s="16" t="n"/>
+      <c r="H44" s="3">
+        <f>1000-F44</f>
+        <v/>
+      </c>
+      <c r="I44" s="16" t="n"/>
+      <c r="J44" s="18">
+        <f>IF(AND(ISNUMBER(E44),ISNUMBER(G44)),G44-E44,"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="18">
+        <f>IF(AND(ISNUMBER(G44),ISNUMBER(I44)),I44-G44,"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="19">
+        <f>IF(AND(ISNUMBER(J44),ISNUMBER(K44)),IF(J44&gt;0,(J44+K44)/J44,""),"")</f>
+        <v/>
+      </c>
+      <c r="M44" s="5" t="n"/>
+      <c r="N44" s="5" t="n"/>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P44" s="17" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>I2-T1</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="11">
+        <f>1000-F45</f>
+        <v/>
+      </c>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="14">
+        <f>IF(AND(ISNUMBER(E45),ISNUMBER(G45)),G45-E45,"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="14">
+        <f>IF(AND(ISNUMBER(G45),ISNUMBER(I45)),I45-G45,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="15">
+        <f>IF(AND(ISNUMBER(J45),ISNUMBER(K45)),IF(J45&gt;0,(J45+K45)/J45,""),"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="20" t="n"/>
+      <c r="N45" s="20" t="n"/>
+      <c r="O45" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>I2-T2</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="n"/>
+      <c r="F46" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G46" s="16" t="n"/>
+      <c r="H46" s="3">
+        <f>1000-F46</f>
+        <v/>
+      </c>
+      <c r="I46" s="16" t="n"/>
+      <c r="J46" s="18">
+        <f>IF(AND(ISNUMBER(E46),ISNUMBER(G46)),G46-E46,"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="18">
+        <f>IF(AND(ISNUMBER(G46),ISNUMBER(I46)),I46-G46,"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="19">
+        <f>IF(AND(ISNUMBER(J46),ISNUMBER(K46)),IF(J46&gt;0,(J46+K46)/J46,""),"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="5" t="n"/>
+      <c r="N46" s="5" t="n"/>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P46" s="17" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>I2-B1</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="3">
+        <f>1000-F47</f>
+        <v/>
+      </c>
+      <c r="I47" s="16" t="n"/>
+      <c r="J47" s="18">
+        <f>IF(AND(ISNUMBER(E47),ISNUMBER(G47)),G47-E47,"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="18">
+        <f>IF(AND(ISNUMBER(G47),ISNUMBER(I47)),I47-G47,"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="19">
+        <f>IF(AND(ISNUMBER(J47),ISNUMBER(K47)),IF(J47&gt;0,(J47+K47)/J47,""),"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="17" t="n"/>
+      <c r="N47" s="17" t="n"/>
+      <c r="O47" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P47" s="17" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>I2-B2</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="n"/>
+      <c r="F48" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G48" s="16" t="n"/>
+      <c r="H48" s="3">
+        <f>1000-F48</f>
+        <v/>
+      </c>
+      <c r="I48" s="16" t="n"/>
+      <c r="J48" s="18">
+        <f>IF(AND(ISNUMBER(E48),ISNUMBER(G48)),G48-E48,"")</f>
+        <v/>
+      </c>
+      <c r="K48" s="18">
+        <f>IF(AND(ISNUMBER(G48),ISNUMBER(I48)),I48-G48,"")</f>
+        <v/>
+      </c>
+      <c r="L48" s="19">
+        <f>IF(AND(ISNUMBER(J48),ISNUMBER(K48)),IF(J48&gt;0,(J48+K48)/J48,""),"")</f>
+        <v/>
+      </c>
+      <c r="M48" s="17" t="n"/>
+      <c r="N48" s="17" t="n"/>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P48" s="17" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>I4-T1</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="11">
+        <f>1000-F49</f>
+        <v/>
+      </c>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="14">
+        <f>IF(AND(ISNUMBER(E49),ISNUMBER(G49)),G49-E49,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="14">
+        <f>IF(AND(ISNUMBER(G49),ISNUMBER(I49)),I49-G49,"")</f>
+        <v/>
+      </c>
+      <c r="L49" s="15">
+        <f>IF(AND(ISNUMBER(J49),ISNUMBER(K49)),IF(J49&gt;0,(J49+K49)/J49,""),"")</f>
+        <v/>
+      </c>
+      <c r="M49" s="20" t="n"/>
+      <c r="N49" s="20" t="n"/>
+      <c r="O49" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P49" s="13" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>I4-T2</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="n"/>
+      <c r="F50" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G50" s="16" t="n"/>
+      <c r="H50" s="3">
+        <f>1000-F50</f>
+        <v/>
+      </c>
+      <c r="I50" s="16" t="n"/>
+      <c r="J50" s="18">
+        <f>IF(AND(ISNUMBER(E50),ISNUMBER(G50)),G50-E50,"")</f>
+        <v/>
+      </c>
+      <c r="K50" s="18">
+        <f>IF(AND(ISNUMBER(G50),ISNUMBER(I50)),I50-G50,"")</f>
+        <v/>
+      </c>
+      <c r="L50" s="19">
+        <f>IF(AND(ISNUMBER(J50),ISNUMBER(K50)),IF(J50&gt;0,(J50+K50)/J50,""),"")</f>
+        <v/>
+      </c>
+      <c r="M50" s="5" t="n"/>
+      <c r="N50" s="5" t="n"/>
+      <c r="O50" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P50" s="17" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>BIN8</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>BIN8-T1</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="11">
+        <f>1000-F51</f>
+        <v/>
+      </c>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="14">
+        <f>IF(AND(ISNUMBER(E51),ISNUMBER(G51)),G51-E51,"")</f>
+        <v/>
+      </c>
+      <c r="K51" s="14">
+        <f>IF(AND(ISNUMBER(G51),ISNUMBER(I51)),I51-G51,"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="15">
+        <f>IF(AND(ISNUMBER(J51),ISNUMBER(K51)),IF(J51&gt;0,(J51+K51)/J51,""),"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="20" t="n"/>
+      <c r="N51" s="20" t="n"/>
+      <c r="O51" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P51" s="13" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>BIN8</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>BIN8-T2</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G52" s="16" t="n"/>
+      <c r="H52" s="3">
+        <f>1000-F52</f>
+        <v/>
+      </c>
+      <c r="I52" s="16" t="n"/>
+      <c r="J52" s="18">
+        <f>IF(AND(ISNUMBER(E52),ISNUMBER(G52)),G52-E52,"")</f>
+        <v/>
+      </c>
+      <c r="K52" s="18">
+        <f>IF(AND(ISNUMBER(G52),ISNUMBER(I52)),I52-G52,"")</f>
+        <v/>
+      </c>
+      <c r="L52" s="19">
+        <f>IF(AND(ISNUMBER(J52),ISNUMBER(K52)),IF(J52&gt;0,(J52+K52)/J52,""),"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="5" t="n"/>
+      <c r="N52" s="5" t="n"/>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P52" s="17" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>BIN8</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>BIN8-B1</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G53" s="16" t="n"/>
+      <c r="H53" s="3">
+        <f>1000-F53</f>
+        <v/>
+      </c>
+      <c r="I53" s="16" t="n"/>
+      <c r="J53" s="18">
+        <f>IF(AND(ISNUMBER(E53),ISNUMBER(G53)),G53-E53,"")</f>
+        <v/>
+      </c>
+      <c r="K53" s="18">
+        <f>IF(AND(ISNUMBER(G53),ISNUMBER(I53)),I53-G53,"")</f>
+        <v/>
+      </c>
+      <c r="L53" s="19">
+        <f>IF(AND(ISNUMBER(J53),ISNUMBER(K53)),IF(J53&gt;0,(J53+K53)/J53,""),"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="17" t="n"/>
+      <c r="N53" s="17" t="n"/>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P53" s="17" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>BIN8</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>BIN8-B2</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G54" s="16" t="n"/>
+      <c r="H54" s="3">
+        <f>1000-F54</f>
+        <v/>
+      </c>
+      <c r="I54" s="16" t="n"/>
+      <c r="J54" s="18">
+        <f>IF(AND(ISNUMBER(E54),ISNUMBER(G54)),G54-E54,"")</f>
+        <v/>
+      </c>
+      <c r="K54" s="18">
+        <f>IF(AND(ISNUMBER(G54),ISNUMBER(I54)),I54-G54,"")</f>
+        <v/>
+      </c>
+      <c r="L54" s="19">
+        <f>IF(AND(ISNUMBER(J54),ISNUMBER(K54)),IF(J54&gt;0,(J54+K54)/J54,""),"")</f>
+        <v/>
+      </c>
+      <c r="M54" s="17" t="n"/>
+      <c r="N54" s="17" t="n"/>
+      <c r="O54" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P54" s="17" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 E49:G49 E50:G50 E51:G51 E52:G52 E53:G53 E54:G54 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48 I49 I50 I51 I52 I53 I54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M29:N29 M30:N30 M33:N33 M34:N34 M39:N39 M40:N40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M29:N29 M30:N30 M39:N39 M40:N40 M47:N47 M48:N48 M53:N53 M54:N54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
data(repeat): round 2 takes BIN8's aqueous phase only (44 vials)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat2_entry.xlsx
+++ b/out/repeat2_entry.xlsx
@@ -299,16 +299,6 @@
         <t>Campaign 1: 1.908 %</t>
       </text>
     </comment>
-    <comment ref="M53" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.6475 %</t>
-      </text>
-    </comment>
-    <comment ref="M54" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.6484 %</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -602,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3217,118 +3207,14 @@
       </c>
       <c r="P52" s="17" t="n"/>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>BIN8-B1</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E53" s="16" t="n"/>
-      <c r="F53" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G53" s="16" t="n"/>
-      <c r="H53" s="3">
-        <f>1000-F53</f>
-        <v/>
-      </c>
-      <c r="I53" s="16" t="n"/>
-      <c r="J53" s="18">
-        <f>IF(AND(ISNUMBER(E53),ISNUMBER(G53)),G53-E53,"")</f>
-        <v/>
-      </c>
-      <c r="K53" s="18">
-        <f>IF(AND(ISNUMBER(G53),ISNUMBER(I53)),I53-G53,"")</f>
-        <v/>
-      </c>
-      <c r="L53" s="19">
-        <f>IF(AND(ISNUMBER(J53),ISNUMBER(K53)),IF(J53&gt;0,(J53+K53)/J53,""),"")</f>
-        <v/>
-      </c>
-      <c r="M53" s="17" t="n"/>
-      <c r="N53" s="17" t="n"/>
-      <c r="O53" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P53" s="17" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>BIN8-B2</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E54" s="16" t="n"/>
-      <c r="F54" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G54" s="16" t="n"/>
-      <c r="H54" s="3">
-        <f>1000-F54</f>
-        <v/>
-      </c>
-      <c r="I54" s="16" t="n"/>
-      <c r="J54" s="18">
-        <f>IF(AND(ISNUMBER(E54),ISNUMBER(G54)),G54-E54,"")</f>
-        <v/>
-      </c>
-      <c r="K54" s="18">
-        <f>IF(AND(ISNUMBER(G54),ISNUMBER(I54)),I54-G54,"")</f>
-        <v/>
-      </c>
-      <c r="L54" s="19">
-        <f>IF(AND(ISNUMBER(J54),ISNUMBER(K54)),IF(J54&gt;0,(J54+K54)/J54,""),"")</f>
-        <v/>
-      </c>
-      <c r="M54" s="17" t="n"/>
-      <c r="N54" s="17" t="n"/>
-      <c r="O54" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P54" s="17" t="n"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 E49:G49 E50:G50 E51:G51 E52:G52 E53:G53 E54:G54 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48 I49 I50 I51 I52 I53 I54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 E49:G49 E50:G50 E51:G51 E52:G52 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48 I49 I50 I51 I52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M29:N29 M30:N30 M39:N39 M40:N40 M47:N47 M48:N48 M53:N53 M54:N54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M29:N29 M30:N30 M39:N39 M40:N40 M47:N47 M48:N48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
data(repeat): BIN1 out of round 2 -- its round-1 repeat is good (user's call)
Round 2 is 13 tubes, 40 vials; A-bin leaves TENTATIVE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat2_entry.xlsx
+++ b/out/repeat2_entry.xlsx
@@ -264,37 +264,22 @@
         <t>Campaign 1: 6.6223 %</t>
       </text>
     </comment>
-    <comment ref="M29" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.5599 %</t>
-      </text>
-    </comment>
-    <comment ref="N29" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.6021 %</t>
-      </text>
-    </comment>
-    <comment ref="M30" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.4736 %</t>
-      </text>
-    </comment>
-    <comment ref="M39" authorId="0" shapeId="0">
+    <comment ref="M35" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.8273 %</t>
       </text>
     </comment>
-    <comment ref="M40" authorId="0" shapeId="0">
+    <comment ref="M36" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.7719 %</t>
       </text>
     </comment>
-    <comment ref="M47" authorId="0" shapeId="0">
+    <comment ref="M43" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.9451 %</t>
       </text>
     </comment>
-    <comment ref="M48" authorId="0" shapeId="0">
+    <comment ref="M44" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.908 %</t>
       </text>
@@ -592,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1962,22 +1947,22 @@
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>BIN1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>BIN1-T1</t>
+          <t>B2-B1</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E29" s="12" t="n"/>
@@ -2002,11 +1987,11 @@
         <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),IF(J29&gt;0,(J29+K29)/J29,""),"")</f>
         <v/>
       </c>
-      <c r="M29" s="13" t="n"/>
-      <c r="N29" s="13" t="n"/>
+      <c r="M29" s="20" t="n"/>
+      <c r="N29" s="20" t="n"/>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P29" s="13" t="n"/>
@@ -2014,22 +1999,22 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>BIN1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>BIN1-T2</t>
+          <t>B2-B2</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E30" s="16" t="n"/>
@@ -2054,76 +2039,76 @@
         <f>IF(AND(ISNUMBER(J30),ISNUMBER(K30)),IF(J30&gt;0,(J30+K30)/J30,""),"")</f>
         <v/>
       </c>
-      <c r="M30" s="17" t="n"/>
-      <c r="N30" s="17" t="n"/>
+      <c r="M30" s="5" t="n"/>
+      <c r="N30" s="5" t="n"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P30" s="17" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>BIN1</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>BIN1-B1</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>B3-B1</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="3">
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="11">
         <f>1000-F31</f>
         <v/>
       </c>
-      <c r="I31" s="16" t="n"/>
-      <c r="J31" s="18">
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="14">
         <f>IF(AND(ISNUMBER(E31),ISNUMBER(G31)),G31-E31,"")</f>
         <v/>
       </c>
-      <c r="K31" s="18">
+      <c r="K31" s="14">
         <f>IF(AND(ISNUMBER(G31),ISNUMBER(I31)),I31-G31,"")</f>
         <v/>
       </c>
-      <c r="L31" s="19">
+      <c r="L31" s="15">
         <f>IF(AND(ISNUMBER(J31),ISNUMBER(K31)),IF(J31&gt;0,(J31+K31)/J31,""),"")</f>
         <v/>
       </c>
-      <c r="M31" s="5" t="n"/>
-      <c r="N31" s="5" t="n"/>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="M31" s="20" t="n"/>
+      <c r="N31" s="20" t="n"/>
+      <c r="O31" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P31" s="17" t="n"/>
+      <c r="P31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>BIN1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>BIN1-B2</t>
+          <t>B3-B2</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2170,12 +2155,12 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>B2-B1</t>
+          <t>B4-B1</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -2222,12 +2207,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>B2-B2</t>
+          <t>B4-B2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2274,22 +2259,22 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>B3-B1</t>
+          <t>F5-T1</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E35" s="12" t="n"/>
@@ -2314,11 +2299,11 @@
         <f>IF(AND(ISNUMBER(J35),ISNUMBER(K35)),IF(J35&gt;0,(J35+K35)/J35,""),"")</f>
         <v/>
       </c>
-      <c r="M35" s="20" t="n"/>
-      <c r="N35" s="20" t="n"/>
+      <c r="M35" s="13" t="n"/>
+      <c r="N35" s="13" t="n"/>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P35" s="13" t="n"/>
@@ -2326,22 +2311,22 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>B3-B2</t>
+          <t>F5-T2</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E36" s="16" t="n"/>
@@ -2366,76 +2351,76 @@
         <f>IF(AND(ISNUMBER(J36),ISNUMBER(K36)),IF(J36&gt;0,(J36+K36)/J36,""),"")</f>
         <v/>
       </c>
-      <c r="M36" s="5" t="n"/>
-      <c r="N36" s="5" t="n"/>
+      <c r="M36" s="17" t="n"/>
+      <c r="N36" s="17" t="n"/>
       <c r="O36" s="3" t="inlineStr">
         <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P36" s="17" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>F5-B1</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G37" s="16" t="n"/>
+      <c r="H37" s="3">
+        <f>1000-F37</f>
+        <v/>
+      </c>
+      <c r="I37" s="16" t="n"/>
+      <c r="J37" s="18">
+        <f>IF(AND(ISNUMBER(E37),ISNUMBER(G37)),G37-E37,"")</f>
+        <v/>
+      </c>
+      <c r="K37" s="18">
+        <f>IF(AND(ISNUMBER(G37),ISNUMBER(I37)),I37-G37,"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="19">
+        <f>IF(AND(ISNUMBER(J37),ISNUMBER(K37)),IF(J37&gt;0,(J37+K37)/J37,""),"")</f>
+        <v/>
+      </c>
+      <c r="M37" s="5" t="n"/>
+      <c r="N37" s="5" t="n"/>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P36" s="17" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>B4-B1</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="n"/>
-      <c r="F37" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G37" s="12" t="n"/>
-      <c r="H37" s="11">
-        <f>1000-F37</f>
-        <v/>
-      </c>
-      <c r="I37" s="12" t="n"/>
-      <c r="J37" s="14">
-        <f>IF(AND(ISNUMBER(E37),ISNUMBER(G37)),G37-E37,"")</f>
-        <v/>
-      </c>
-      <c r="K37" s="14">
-        <f>IF(AND(ISNUMBER(G37),ISNUMBER(I37)),I37-G37,"")</f>
-        <v/>
-      </c>
-      <c r="L37" s="15">
-        <f>IF(AND(ISNUMBER(J37),ISNUMBER(K37)),IF(J37&gt;0,(J37+K37)/J37,""),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="20" t="n"/>
-      <c r="N37" s="20" t="n"/>
-      <c r="O37" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P37" s="13" t="n"/>
+      <c r="P37" s="17" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>B4-B2</t>
+          <t>F5-B2</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2482,22 +2467,22 @@
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>F5-T1</t>
+          <t>BIN6-B1</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E39" s="12" t="n"/>
@@ -2522,11 +2507,11 @@
         <f>IF(AND(ISNUMBER(J39),ISNUMBER(K39)),IF(J39&gt;0,(J39+K39)/J39,""),"")</f>
         <v/>
       </c>
-      <c r="M39" s="13" t="n"/>
-      <c r="N39" s="13" t="n"/>
+      <c r="M39" s="20" t="n"/>
+      <c r="N39" s="20" t="n"/>
       <c r="O39" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P39" s="13" t="n"/>
@@ -2534,22 +2519,22 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>F5-T2</t>
+          <t>BIN6-B2</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E40" s="16" t="n"/>
@@ -2574,81 +2559,81 @@
         <f>IF(AND(ISNUMBER(J40),ISNUMBER(K40)),IF(J40&gt;0,(J40+K40)/J40,""),"")</f>
         <v/>
       </c>
-      <c r="M40" s="17" t="n"/>
-      <c r="N40" s="17" t="n"/>
+      <c r="M40" s="5" t="n"/>
+      <c r="N40" s="5" t="n"/>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>F5-B1</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>I2-T1</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="3">
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41" s="11">
         <f>1000-F41</f>
         <v/>
       </c>
-      <c r="I41" s="16" t="n"/>
-      <c r="J41" s="18">
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="14">
         <f>IF(AND(ISNUMBER(E41),ISNUMBER(G41)),G41-E41,"")</f>
         <v/>
       </c>
-      <c r="K41" s="18">
+      <c r="K41" s="14">
         <f>IF(AND(ISNUMBER(G41),ISNUMBER(I41)),I41-G41,"")</f>
         <v/>
       </c>
-      <c r="L41" s="19">
+      <c r="L41" s="15">
         <f>IF(AND(ISNUMBER(J41),ISNUMBER(K41)),IF(J41&gt;0,(J41+K41)/J41,""),"")</f>
         <v/>
       </c>
-      <c r="M41" s="5" t="n"/>
-      <c r="N41" s="5" t="n"/>
-      <c r="O41" s="3" t="inlineStr">
+      <c r="M41" s="20" t="n"/>
+      <c r="N41" s="20" t="n"/>
+      <c r="O41" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P41" s="17" t="n"/>
+      <c r="P41" s="13" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>F5-B2</t>
+          <t>I2-T2</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -2688,66 +2673,66 @@
       <c r="P42" s="17" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>BIN6</t>
-        </is>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>BIN6-B1</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>I2-B1</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D43" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="n"/>
-      <c r="F43" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G43" s="12" t="n"/>
-      <c r="H43" s="11">
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>organic</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="n"/>
+      <c r="F43" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G43" s="16" t="n"/>
+      <c r="H43" s="3">
         <f>1000-F43</f>
         <v/>
       </c>
-      <c r="I43" s="12" t="n"/>
-      <c r="J43" s="14">
+      <c r="I43" s="16" t="n"/>
+      <c r="J43" s="18">
         <f>IF(AND(ISNUMBER(E43),ISNUMBER(G43)),G43-E43,"")</f>
         <v/>
       </c>
-      <c r="K43" s="14">
+      <c r="K43" s="18">
         <f>IF(AND(ISNUMBER(G43),ISNUMBER(I43)),I43-G43,"")</f>
         <v/>
       </c>
-      <c r="L43" s="15">
+      <c r="L43" s="19">
         <f>IF(AND(ISNUMBER(J43),ISNUMBER(K43)),IF(J43&gt;0,(J43+K43)/J43,""),"")</f>
         <v/>
       </c>
-      <c r="M43" s="20" t="n"/>
-      <c r="N43" s="20" t="n"/>
-      <c r="O43" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P43" s="13" t="n"/>
+      <c r="M43" s="17" t="n"/>
+      <c r="N43" s="17" t="n"/>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>fresh: type the new KF</t>
+        </is>
+      </c>
+      <c r="P43" s="17" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>BIN6</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>BIN6-B2</t>
+          <t>I2-B2</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2757,7 +2742,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E44" s="16" t="n"/>
@@ -2782,11 +2767,11 @@
         <f>IF(AND(ISNUMBER(J44),ISNUMBER(K44)),IF(J44&gt;0,(J44+K44)/J44,""),"")</f>
         <v/>
       </c>
-      <c r="M44" s="5" t="n"/>
-      <c r="N44" s="5" t="n"/>
+      <c r="M44" s="17" t="n"/>
+      <c r="N44" s="17" t="n"/>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P44" s="17" t="n"/>
@@ -2794,12 +2779,12 @@
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>I2-T1</t>
+          <t>I4-T1</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
@@ -2846,12 +2831,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>I2-T2</t>
+          <t>I4-T2</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2896,76 +2881,76 @@
       <c r="P46" s="17" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>I2-B1</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E47" s="16" t="n"/>
-      <c r="F47" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="3">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>BIN8</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>BIN8-T1</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="11">
         <f>1000-F47</f>
         <v/>
       </c>
-      <c r="I47" s="16" t="n"/>
-      <c r="J47" s="18">
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="14">
         <f>IF(AND(ISNUMBER(E47),ISNUMBER(G47)),G47-E47,"")</f>
         <v/>
       </c>
-      <c r="K47" s="18">
+      <c r="K47" s="14">
         <f>IF(AND(ISNUMBER(G47),ISNUMBER(I47)),I47-G47,"")</f>
         <v/>
       </c>
-      <c r="L47" s="19">
+      <c r="L47" s="15">
         <f>IF(AND(ISNUMBER(J47),ISNUMBER(K47)),IF(J47&gt;0,(J47+K47)/J47,""),"")</f>
         <v/>
       </c>
-      <c r="M47" s="17" t="n"/>
-      <c r="N47" s="17" t="n"/>
-      <c r="O47" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P47" s="17" t="n"/>
+      <c r="M47" s="20" t="n"/>
+      <c r="N47" s="20" t="n"/>
+      <c r="O47" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P47" s="13" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>BIN8</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>I2-B2</t>
+          <t>BIN8-T2</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E48" s="16" t="n"/>
@@ -2990,231 +2975,23 @@
         <f>IF(AND(ISNUMBER(J48),ISNUMBER(K48)),IF(J48&gt;0,(J48+K48)/J48,""),"")</f>
         <v/>
       </c>
-      <c r="M48" s="17" t="n"/>
-      <c r="N48" s="17" t="n"/>
+      <c r="M48" s="5" t="n"/>
+      <c r="N48" s="5" t="n"/>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P48" s="17" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B49" s="11" t="inlineStr">
-        <is>
-          <t>I4-T1</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="n"/>
-      <c r="F49" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G49" s="12" t="n"/>
-      <c r="H49" s="11">
-        <f>1000-F49</f>
-        <v/>
-      </c>
-      <c r="I49" s="12" t="n"/>
-      <c r="J49" s="14">
-        <f>IF(AND(ISNUMBER(E49),ISNUMBER(G49)),G49-E49,"")</f>
-        <v/>
-      </c>
-      <c r="K49" s="14">
-        <f>IF(AND(ISNUMBER(G49),ISNUMBER(I49)),I49-G49,"")</f>
-        <v/>
-      </c>
-      <c r="L49" s="15">
-        <f>IF(AND(ISNUMBER(J49),ISNUMBER(K49)),IF(J49&gt;0,(J49+K49)/J49,""),"")</f>
-        <v/>
-      </c>
-      <c r="M49" s="20" t="n"/>
-      <c r="N49" s="20" t="n"/>
-      <c r="O49" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P49" s="13" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>I4-T2</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E50" s="16" t="n"/>
-      <c r="F50" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G50" s="16" t="n"/>
-      <c r="H50" s="3">
-        <f>1000-F50</f>
-        <v/>
-      </c>
-      <c r="I50" s="16" t="n"/>
-      <c r="J50" s="18">
-        <f>IF(AND(ISNUMBER(E50),ISNUMBER(G50)),G50-E50,"")</f>
-        <v/>
-      </c>
-      <c r="K50" s="18">
-        <f>IF(AND(ISNUMBER(G50),ISNUMBER(I50)),I50-G50,"")</f>
-        <v/>
-      </c>
-      <c r="L50" s="19">
-        <f>IF(AND(ISNUMBER(J50),ISNUMBER(K50)),IF(J50&gt;0,(J50+K50)/J50,""),"")</f>
-        <v/>
-      </c>
-      <c r="M50" s="5" t="n"/>
-      <c r="N50" s="5" t="n"/>
-      <c r="O50" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P50" s="17" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>BIN8-T1</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E51" s="12" t="n"/>
-      <c r="F51" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G51" s="12" t="n"/>
-      <c r="H51" s="11">
-        <f>1000-F51</f>
-        <v/>
-      </c>
-      <c r="I51" s="12" t="n"/>
-      <c r="J51" s="14">
-        <f>IF(AND(ISNUMBER(E51),ISNUMBER(G51)),G51-E51,"")</f>
-        <v/>
-      </c>
-      <c r="K51" s="14">
-        <f>IF(AND(ISNUMBER(G51),ISNUMBER(I51)),I51-G51,"")</f>
-        <v/>
-      </c>
-      <c r="L51" s="15">
-        <f>IF(AND(ISNUMBER(J51),ISNUMBER(K51)),IF(J51&gt;0,(J51+K51)/J51,""),"")</f>
-        <v/>
-      </c>
-      <c r="M51" s="20" t="n"/>
-      <c r="N51" s="20" t="n"/>
-      <c r="O51" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P51" s="13" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>BIN8-T2</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G52" s="16" t="n"/>
-      <c r="H52" s="3">
-        <f>1000-F52</f>
-        <v/>
-      </c>
-      <c r="I52" s="16" t="n"/>
-      <c r="J52" s="18">
-        <f>IF(AND(ISNUMBER(E52),ISNUMBER(G52)),G52-E52,"")</f>
-        <v/>
-      </c>
-      <c r="K52" s="18">
-        <f>IF(AND(ISNUMBER(G52),ISNUMBER(I52)),I52-G52,"")</f>
-        <v/>
-      </c>
-      <c r="L52" s="19">
-        <f>IF(AND(ISNUMBER(J52),ISNUMBER(K52)),IF(J52&gt;0,(J52+K52)/J52,""),"")</f>
-        <v/>
-      </c>
-      <c r="M52" s="5" t="n"/>
-      <c r="N52" s="5" t="n"/>
-      <c r="O52" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P52" s="17" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 E49:G49 E50:G50 E51:G51 E52:G52 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48 I49 I50 I51 I52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M29:N29 M30:N30 M39:N39 M40:N40 M47:N47 M48:N48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M35:N35 M36:N36 M43:N43 M44:N44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
data(repeat): tighten round 2 to A1 A4 A5 F5 I2 + B2 B3 B4 BIN6 (aq)
A2, A3, I4 and BIN8 leave round 2 and TENTATIVE: final as they stand (user's call). A5
is the aqueous endpoint with 4x the binary's terpene at the 2PE-rich end. 9 tubes,
28 vials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat2_entry.xlsx
+++ b/out/repeat2_entry.xlsx
@@ -219,67 +219,42 @@
         <t>Campaign 1: 1.968 %</t>
       </text>
     </comment>
-    <comment ref="M15" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 8.5693 %</t>
-      </text>
-    </comment>
-    <comment ref="N15" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 8.5126 %</t>
-      </text>
-    </comment>
-    <comment ref="N16" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 8.5203 %</t>
-      </text>
-    </comment>
-    <comment ref="M17" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 4.0063 %</t>
-      </text>
-    </comment>
-    <comment ref="M18" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 4.049 %</t>
-      </text>
-    </comment>
-    <comment ref="M21" authorId="0" shapeId="0">
+    <comment ref="M13" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.6416 %</t>
       </text>
     </comment>
-    <comment ref="M22" authorId="0" shapeId="0">
+    <comment ref="M14" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.6825 %</t>
       </text>
     </comment>
-    <comment ref="M27" authorId="0" shapeId="0">
+    <comment ref="M19" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 6.6554 %</t>
       </text>
     </comment>
-    <comment ref="M28" authorId="0" shapeId="0">
+    <comment ref="M20" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 6.6223 %</t>
       </text>
     </comment>
-    <comment ref="M35" authorId="0" shapeId="0">
+    <comment ref="M27" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.8273 %</t>
       </text>
     </comment>
-    <comment ref="M36" authorId="0" shapeId="0">
+    <comment ref="M28" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 2.7719 %</t>
       </text>
     </comment>
-    <comment ref="M43" authorId="0" shapeId="0">
+    <comment ref="M35" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.9451 %</t>
       </text>
     </comment>
-    <comment ref="M44" authorId="0" shapeId="0">
+    <comment ref="M36" authorId="0" shapeId="0">
       <text>
         <t>Campaign 1: 1.908 %</t>
       </text>
@@ -577,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1115,12 +1090,12 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>A2-T1</t>
+          <t>A4-T1</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -1130,7 +1105,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E13" s="12" t="n"/>
@@ -1155,11 +1130,11 @@
         <f>IF(AND(ISNUMBER(J13),ISNUMBER(K13)),IF(J13&gt;0,(J13+K13)/J13,""),"")</f>
         <v/>
       </c>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="n"/>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P13" s="13" t="n"/>
@@ -1167,12 +1142,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>A2-T2</t>
+          <t>A4-T2</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1182,7 +1157,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E14" s="16" t="n"/>
@@ -1207,11 +1182,11 @@
         <f>IF(AND(ISNUMBER(J14),ISNUMBER(K14)),IF(J14&gt;0,(J14+K14)/J14,""),"")</f>
         <v/>
       </c>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="17" t="n"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P14" s="17" t="n"/>
@@ -1219,12 +1194,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>A2-B1</t>
+          <t>A4-B1</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1234,7 +1209,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E15" s="16" t="n"/>
@@ -1259,11 +1234,11 @@
         <f>IF(AND(ISNUMBER(J15),ISNUMBER(K15)),IF(J15&gt;0,(J15+K15)/J15,""),"")</f>
         <v/>
       </c>
-      <c r="M15" s="17" t="n"/>
-      <c r="N15" s="17" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P15" s="17" t="n"/>
@@ -1271,12 +1246,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>A2-B2</t>
+          <t>A4-B2</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1286,7 +1261,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E16" s="16" t="n"/>
@@ -1311,11 +1286,11 @@
         <f>IF(AND(ISNUMBER(J16),ISNUMBER(K16)),IF(J16&gt;0,(J16+K16)/J16,""),"")</f>
         <v/>
       </c>
-      <c r="M16" s="17" t="n"/>
-      <c r="N16" s="17" t="n"/>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P16" s="17" t="n"/>
@@ -1323,12 +1298,12 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>A3-T1</t>
+          <t>A5-T1</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -1338,7 +1313,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E17" s="12" t="n"/>
@@ -1363,11 +1338,11 @@
         <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),IF(J17&gt;0,(J17+K17)/J17,""),"")</f>
         <v/>
       </c>
-      <c r="M17" s="13" t="n"/>
-      <c r="N17" s="13" t="n"/>
+      <c r="M17" s="20" t="n"/>
+      <c r="N17" s="20" t="n"/>
       <c r="O17" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P17" s="13" t="n"/>
@@ -1375,12 +1350,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>A3-T2</t>
+          <t>A5-T2</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1390,7 +1365,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E18" s="16" t="n"/>
@@ -1415,11 +1390,11 @@
         <f>IF(AND(ISNUMBER(J18),ISNUMBER(K18)),IF(J18&gt;0,(J18+K18)/J18,""),"")</f>
         <v/>
       </c>
-      <c r="M18" s="17" t="n"/>
-      <c r="N18" s="17" t="n"/>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="n"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P18" s="17" t="n"/>
@@ -1427,12 +1402,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>A3-B1</t>
+          <t>A5-B1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1442,7 +1417,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E19" s="16" t="n"/>
@@ -1467,11 +1442,11 @@
         <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
         <v/>
       </c>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5" t="n"/>
+      <c r="M19" s="17" t="n"/>
+      <c r="N19" s="17" t="n"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P19" s="17" t="n"/>
@@ -1479,12 +1454,12 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>A3-B2</t>
+          <t>A5-B2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1494,7 +1469,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>aqueous</t>
+          <t>organic</t>
         </is>
       </c>
       <c r="E20" s="16" t="n"/>
@@ -1519,11 +1494,11 @@
         <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
         <v/>
       </c>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="n"/>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>n/a: by difference</t>
+          <t>fresh: type the new KF</t>
         </is>
       </c>
       <c r="P20" s="17" t="n"/>
@@ -1531,22 +1506,22 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>A4-T1</t>
+          <t>B2-B1</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E21" s="12" t="n"/>
@@ -1571,11 +1546,11 @@
         <f>IF(AND(ISNUMBER(J21),ISNUMBER(K21)),IF(J21&gt;0,(J21+K21)/J21,""),"")</f>
         <v/>
       </c>
-      <c r="M21" s="13" t="n"/>
-      <c r="N21" s="13" t="n"/>
+      <c r="M21" s="20" t="n"/>
+      <c r="N21" s="20" t="n"/>
       <c r="O21" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P21" s="13" t="n"/>
@@ -1583,22 +1558,22 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>A4-T2</t>
+          <t>B2-B2</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E22" s="16" t="n"/>
@@ -1623,76 +1598,76 @@
         <f>IF(AND(ISNUMBER(J22),ISNUMBER(K22)),IF(J22&gt;0,(J22+K22)/J22,""),"")</f>
         <v/>
       </c>
-      <c r="M22" s="17" t="n"/>
-      <c r="N22" s="17" t="n"/>
+      <c r="M22" s="5" t="n"/>
+      <c r="N22" s="5" t="n"/>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>A4</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>A4-B1</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>B3-B1</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="3">
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="11">
         <f>1000-F23</f>
         <v/>
       </c>
-      <c r="I23" s="16" t="n"/>
-      <c r="J23" s="18">
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="14">
         <f>IF(AND(ISNUMBER(E23),ISNUMBER(G23)),G23-E23,"")</f>
         <v/>
       </c>
-      <c r="K23" s="18">
+      <c r="K23" s="14">
         <f>IF(AND(ISNUMBER(G23),ISNUMBER(I23)),I23-G23,"")</f>
         <v/>
       </c>
-      <c r="L23" s="19">
+      <c r="L23" s="15">
         <f>IF(AND(ISNUMBER(J23),ISNUMBER(K23)),IF(J23&gt;0,(J23+K23)/J23,""),"")</f>
         <v/>
       </c>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="3" t="inlineStr">
+      <c r="M23" s="20" t="n"/>
+      <c r="N23" s="20" t="n"/>
+      <c r="O23" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P23" s="17" t="n"/>
+      <c r="P23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>A4-B2</t>
+          <t>B3-B2</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1739,17 +1714,17 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>A5-T1</t>
+          <t>B4-B1</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1791,17 +1766,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>A5-T2</t>
+          <t>B4-B2</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1841,71 +1816,71 @@
       <c r="P26" s="17" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>A5-B1</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>F5-T1</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Superior</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>organic</t>
         </is>
       </c>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="3">
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="11">
         <f>1000-F27</f>
         <v/>
       </c>
-      <c r="I27" s="16" t="n"/>
-      <c r="J27" s="18">
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="14">
         <f>IF(AND(ISNUMBER(E27),ISNUMBER(G27)),G27-E27,"")</f>
         <v/>
       </c>
-      <c r="K27" s="18">
+      <c r="K27" s="14">
         <f>IF(AND(ISNUMBER(G27),ISNUMBER(I27)),I27-G27,"")</f>
         <v/>
       </c>
-      <c r="L27" s="19">
+      <c r="L27" s="15">
         <f>IF(AND(ISNUMBER(J27),ISNUMBER(K27)),IF(J27&gt;0,(J27+K27)/J27,""),"")</f>
         <v/>
       </c>
-      <c r="M27" s="17" t="n"/>
-      <c r="N27" s="17" t="n"/>
-      <c r="O27" s="3" t="inlineStr">
+      <c r="M27" s="13" t="n"/>
+      <c r="N27" s="13" t="n"/>
+      <c r="O27" s="11" t="inlineStr">
         <is>
           <t>fresh: type the new KF</t>
         </is>
       </c>
-      <c r="P27" s="17" t="n"/>
+      <c r="P27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>A5-B2</t>
+          <t>F5-T2</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1945,66 +1920,66 @@
       <c r="P28" s="17" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>B2-B1</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>F5-B1</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="11">
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="3">
         <f>1000-F29</f>
         <v/>
       </c>
-      <c r="I29" s="12" t="n"/>
-      <c r="J29" s="14">
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="18">
         <f>IF(AND(ISNUMBER(E29),ISNUMBER(G29)),G29-E29,"")</f>
         <v/>
       </c>
-      <c r="K29" s="14">
+      <c r="K29" s="18">
         <f>IF(AND(ISNUMBER(G29),ISNUMBER(I29)),I29-G29,"")</f>
         <v/>
       </c>
-      <c r="L29" s="15">
+      <c r="L29" s="19">
         <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),IF(J29&gt;0,(J29+K29)/J29,""),"")</f>
         <v/>
       </c>
-      <c r="M29" s="20" t="n"/>
-      <c r="N29" s="20" t="n"/>
-      <c r="O29" s="11" t="inlineStr">
+      <c r="M29" s="5" t="n"/>
+      <c r="N29" s="5" t="n"/>
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P29" s="13" t="n"/>
+      <c r="P29" s="17" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>B2-B2</t>
+          <t>F5-B2</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2051,12 +2026,12 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>B3-B1</t>
+          <t>BIN6-B1</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -2103,12 +2078,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>B3-B2</t>
+          <t>BIN6-B2</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2155,17 +2130,17 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>B4-B1</t>
+          <t>I2-T1</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -2207,17 +2182,17 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>B4-B2</t>
+          <t>I2-T2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2257,71 +2232,71 @@
       <c r="P34" s="17" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>F5-T1</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>I2-B1</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Inferior</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>organic</t>
         </is>
       </c>
-      <c r="E35" s="12" t="n"/>
-      <c r="F35" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="11">
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="G35" s="16" t="n"/>
+      <c r="H35" s="3">
         <f>1000-F35</f>
         <v/>
       </c>
-      <c r="I35" s="12" t="n"/>
-      <c r="J35" s="14">
+      <c r="I35" s="16" t="n"/>
+      <c r="J35" s="18">
         <f>IF(AND(ISNUMBER(E35),ISNUMBER(G35)),G35-E35,"")</f>
         <v/>
       </c>
-      <c r="K35" s="14">
+      <c r="K35" s="18">
         <f>IF(AND(ISNUMBER(G35),ISNUMBER(I35)),I35-G35,"")</f>
         <v/>
       </c>
-      <c r="L35" s="15">
+      <c r="L35" s="19">
         <f>IF(AND(ISNUMBER(J35),ISNUMBER(K35)),IF(J35&gt;0,(J35+K35)/J35,""),"")</f>
         <v/>
       </c>
-      <c r="M35" s="13" t="n"/>
-      <c r="N35" s="13" t="n"/>
-      <c r="O35" s="11" t="inlineStr">
+      <c r="M35" s="17" t="n"/>
+      <c r="N35" s="17" t="n"/>
+      <c r="O35" s="3" t="inlineStr">
         <is>
           <t>fresh: type the new KF</t>
         </is>
       </c>
-      <c r="P35" s="13" t="n"/>
+      <c r="P35" s="17" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>F5</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>F5-T2</t>
+          <t>I2-B2</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2360,638 +2335,14 @@
       </c>
       <c r="P36" s="17" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>F5-B1</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="3">
-        <f>1000-F37</f>
-        <v/>
-      </c>
-      <c r="I37" s="16" t="n"/>
-      <c r="J37" s="18">
-        <f>IF(AND(ISNUMBER(E37),ISNUMBER(G37)),G37-E37,"")</f>
-        <v/>
-      </c>
-      <c r="K37" s="18">
-        <f>IF(AND(ISNUMBER(G37),ISNUMBER(I37)),I37-G37,"")</f>
-        <v/>
-      </c>
-      <c r="L37" s="19">
-        <f>IF(AND(ISNUMBER(J37),ISNUMBER(K37)),IF(J37&gt;0,(J37+K37)/J37,""),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="5" t="n"/>
-      <c r="N37" s="5" t="n"/>
-      <c r="O37" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P37" s="17" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>F5-B2</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="3">
-        <f>1000-F38</f>
-        <v/>
-      </c>
-      <c r="I38" s="16" t="n"/>
-      <c r="J38" s="18">
-        <f>IF(AND(ISNUMBER(E38),ISNUMBER(G38)),G38-E38,"")</f>
-        <v/>
-      </c>
-      <c r="K38" s="18">
-        <f>IF(AND(ISNUMBER(G38),ISNUMBER(I38)),I38-G38,"")</f>
-        <v/>
-      </c>
-      <c r="L38" s="19">
-        <f>IF(AND(ISNUMBER(J38),ISNUMBER(K38)),IF(J38&gt;0,(J38+K38)/J38,""),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="5" t="n"/>
-      <c r="N38" s="5" t="n"/>
-      <c r="O38" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P38" s="17" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>BIN6</t>
-        </is>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>BIN6-B1</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="n"/>
-      <c r="F39" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G39" s="12" t="n"/>
-      <c r="H39" s="11">
-        <f>1000-F39</f>
-        <v/>
-      </c>
-      <c r="I39" s="12" t="n"/>
-      <c r="J39" s="14">
-        <f>IF(AND(ISNUMBER(E39),ISNUMBER(G39)),G39-E39,"")</f>
-        <v/>
-      </c>
-      <c r="K39" s="14">
-        <f>IF(AND(ISNUMBER(G39),ISNUMBER(I39)),I39-G39,"")</f>
-        <v/>
-      </c>
-      <c r="L39" s="15">
-        <f>IF(AND(ISNUMBER(J39),ISNUMBER(K39)),IF(J39&gt;0,(J39+K39)/J39,""),"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="20" t="n"/>
-      <c r="N39" s="20" t="n"/>
-      <c r="O39" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P39" s="13" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>BIN6</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>BIN6-B2</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="3">
-        <f>1000-F40</f>
-        <v/>
-      </c>
-      <c r="I40" s="16" t="n"/>
-      <c r="J40" s="18">
-        <f>IF(AND(ISNUMBER(E40),ISNUMBER(G40)),G40-E40,"")</f>
-        <v/>
-      </c>
-      <c r="K40" s="18">
-        <f>IF(AND(ISNUMBER(G40),ISNUMBER(I40)),I40-G40,"")</f>
-        <v/>
-      </c>
-      <c r="L40" s="19">
-        <f>IF(AND(ISNUMBER(J40),ISNUMBER(K40)),IF(J40&gt;0,(J40+K40)/J40,""),"")</f>
-        <v/>
-      </c>
-      <c r="M40" s="5" t="n"/>
-      <c r="N40" s="5" t="n"/>
-      <c r="O40" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P40" s="17" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>I2-T1</t>
-        </is>
-      </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G41" s="12" t="n"/>
-      <c r="H41" s="11">
-        <f>1000-F41</f>
-        <v/>
-      </c>
-      <c r="I41" s="12" t="n"/>
-      <c r="J41" s="14">
-        <f>IF(AND(ISNUMBER(E41),ISNUMBER(G41)),G41-E41,"")</f>
-        <v/>
-      </c>
-      <c r="K41" s="14">
-        <f>IF(AND(ISNUMBER(G41),ISNUMBER(I41)),I41-G41,"")</f>
-        <v/>
-      </c>
-      <c r="L41" s="15">
-        <f>IF(AND(ISNUMBER(J41),ISNUMBER(K41)),IF(J41&gt;0,(J41+K41)/J41,""),"")</f>
-        <v/>
-      </c>
-      <c r="M41" s="20" t="n"/>
-      <c r="N41" s="20" t="n"/>
-      <c r="O41" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P41" s="13" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>I2-T2</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E42" s="16" t="n"/>
-      <c r="F42" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G42" s="16" t="n"/>
-      <c r="H42" s="3">
-        <f>1000-F42</f>
-        <v/>
-      </c>
-      <c r="I42" s="16" t="n"/>
-      <c r="J42" s="18">
-        <f>IF(AND(ISNUMBER(E42),ISNUMBER(G42)),G42-E42,"")</f>
-        <v/>
-      </c>
-      <c r="K42" s="18">
-        <f>IF(AND(ISNUMBER(G42),ISNUMBER(I42)),I42-G42,"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="19">
-        <f>IF(AND(ISNUMBER(J42),ISNUMBER(K42)),IF(J42&gt;0,(J42+K42)/J42,""),"")</f>
-        <v/>
-      </c>
-      <c r="M42" s="5" t="n"/>
-      <c r="N42" s="5" t="n"/>
-      <c r="O42" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P42" s="17" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>I2-B1</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G43" s="16" t="n"/>
-      <c r="H43" s="3">
-        <f>1000-F43</f>
-        <v/>
-      </c>
-      <c r="I43" s="16" t="n"/>
-      <c r="J43" s="18">
-        <f>IF(AND(ISNUMBER(E43),ISNUMBER(G43)),G43-E43,"")</f>
-        <v/>
-      </c>
-      <c r="K43" s="18">
-        <f>IF(AND(ISNUMBER(G43),ISNUMBER(I43)),I43-G43,"")</f>
-        <v/>
-      </c>
-      <c r="L43" s="19">
-        <f>IF(AND(ISNUMBER(J43),ISNUMBER(K43)),IF(J43&gt;0,(J43+K43)/J43,""),"")</f>
-        <v/>
-      </c>
-      <c r="M43" s="17" t="n"/>
-      <c r="N43" s="17" t="n"/>
-      <c r="O43" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P43" s="17" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>I2-B2</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E44" s="16" t="n"/>
-      <c r="F44" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G44" s="16" t="n"/>
-      <c r="H44" s="3">
-        <f>1000-F44</f>
-        <v/>
-      </c>
-      <c r="I44" s="16" t="n"/>
-      <c r="J44" s="18">
-        <f>IF(AND(ISNUMBER(E44),ISNUMBER(G44)),G44-E44,"")</f>
-        <v/>
-      </c>
-      <c r="K44" s="18">
-        <f>IF(AND(ISNUMBER(G44),ISNUMBER(I44)),I44-G44,"")</f>
-        <v/>
-      </c>
-      <c r="L44" s="19">
-        <f>IF(AND(ISNUMBER(J44),ISNUMBER(K44)),IF(J44&gt;0,(J44+K44)/J44,""),"")</f>
-        <v/>
-      </c>
-      <c r="M44" s="17" t="n"/>
-      <c r="N44" s="17" t="n"/>
-      <c r="O44" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P44" s="17" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>I4-T1</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="n"/>
-      <c r="F45" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G45" s="12" t="n"/>
-      <c r="H45" s="11">
-        <f>1000-F45</f>
-        <v/>
-      </c>
-      <c r="I45" s="12" t="n"/>
-      <c r="J45" s="14">
-        <f>IF(AND(ISNUMBER(E45),ISNUMBER(G45)),G45-E45,"")</f>
-        <v/>
-      </c>
-      <c r="K45" s="14">
-        <f>IF(AND(ISNUMBER(G45),ISNUMBER(I45)),I45-G45,"")</f>
-        <v/>
-      </c>
-      <c r="L45" s="15">
-        <f>IF(AND(ISNUMBER(J45),ISNUMBER(K45)),IF(J45&gt;0,(J45+K45)/J45,""),"")</f>
-        <v/>
-      </c>
-      <c r="M45" s="20" t="n"/>
-      <c r="N45" s="20" t="n"/>
-      <c r="O45" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P45" s="13" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>I4-T2</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E46" s="16" t="n"/>
-      <c r="F46" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G46" s="16" t="n"/>
-      <c r="H46" s="3">
-        <f>1000-F46</f>
-        <v/>
-      </c>
-      <c r="I46" s="16" t="n"/>
-      <c r="J46" s="18">
-        <f>IF(AND(ISNUMBER(E46),ISNUMBER(G46)),G46-E46,"")</f>
-        <v/>
-      </c>
-      <c r="K46" s="18">
-        <f>IF(AND(ISNUMBER(G46),ISNUMBER(I46)),I46-G46,"")</f>
-        <v/>
-      </c>
-      <c r="L46" s="19">
-        <f>IF(AND(ISNUMBER(J46),ISNUMBER(K46)),IF(J46&gt;0,(J46+K46)/J46,""),"")</f>
-        <v/>
-      </c>
-      <c r="M46" s="5" t="n"/>
-      <c r="N46" s="5" t="n"/>
-      <c r="O46" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P46" s="17" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="11" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B47" s="11" t="inlineStr">
-        <is>
-          <t>BIN8-T1</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D47" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="11">
-        <f>1000-F47</f>
-        <v/>
-      </c>
-      <c r="I47" s="12" t="n"/>
-      <c r="J47" s="14">
-        <f>IF(AND(ISNUMBER(E47),ISNUMBER(G47)),G47-E47,"")</f>
-        <v/>
-      </c>
-      <c r="K47" s="14">
-        <f>IF(AND(ISNUMBER(G47),ISNUMBER(I47)),I47-G47,"")</f>
-        <v/>
-      </c>
-      <c r="L47" s="15">
-        <f>IF(AND(ISNUMBER(J47),ISNUMBER(K47)),IF(J47&gt;0,(J47+K47)/J47,""),"")</f>
-        <v/>
-      </c>
-      <c r="M47" s="20" t="n"/>
-      <c r="N47" s="20" t="n"/>
-      <c r="O47" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P47" s="13" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>BIN8</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>BIN8-T2</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E48" s="16" t="n"/>
-      <c r="F48" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G48" s="16" t="n"/>
-      <c r="H48" s="3">
-        <f>1000-F48</f>
-        <v/>
-      </c>
-      <c r="I48" s="16" t="n"/>
-      <c r="J48" s="18">
-        <f>IF(AND(ISNUMBER(E48),ISNUMBER(G48)),G48-E48,"")</f>
-        <v/>
-      </c>
-      <c r="K48" s="18">
-        <f>IF(AND(ISNUMBER(G48),ISNUMBER(I48)),I48-G48,"")</f>
-        <v/>
-      </c>
-      <c r="L48" s="19">
-        <f>IF(AND(ISNUMBER(J48),ISNUMBER(K48)),IF(J48&gt;0,(J48+K48)/J48,""),"")</f>
-        <v/>
-      </c>
-      <c r="M48" s="5" t="n"/>
-      <c r="N48" s="5" t="n"/>
-      <c r="O48" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P48" s="17" t="n"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 E37:G37 E38:G38 E39:G39 E40:G40 E41:G41 E42:G42 E43:G43 E44:G44 E45:G45 E46:G46 E47:G47 E48:G48 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M15:N15 M16:N16 M17:N17 M18:N18 M21:N21 M22:N22 M27:N27 M28:N28 M35:N35 M36:N36 M43:N43 M44:N44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M19:N19 M20:N20 M27:N27 M28:N28 M35:N35 M36:N36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(repeat): round 2 samples aqueous vials only; the vial sheet hides organic rows
The user recycles every tube's campaign-1 organic phase and KF, so all nine round-2 tubes
are ':aq' (18 vials). An aqueous-only tube's organic rows are now hidden on the printed
vial sheet (campaign-1 KF decides which phase that is: campaign1_kf/organic_phase move
into make_repeat_workbook, make_entry_workbook imports them).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat2_entry.xlsx
+++ b/out/repeat2_entry.xlsx
@@ -118,6 +118,7 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -126,7 +127,6 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -201,66 +201,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>make_entry_workbook</author>
-  </authors>
-  <commentList>
-    <comment ref="M9" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.9303 %</t>
-      </text>
-    </comment>
-    <comment ref="M10" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.968 %</t>
-      </text>
-    </comment>
-    <comment ref="M13" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 2.6416 %</t>
-      </text>
-    </comment>
-    <comment ref="M14" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 2.6825 %</t>
-      </text>
-    </comment>
-    <comment ref="M19" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 6.6554 %</t>
-      </text>
-    </comment>
-    <comment ref="M20" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 6.6223 %</t>
-      </text>
-    </comment>
-    <comment ref="M27" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 2.8273 %</t>
-      </text>
-    </comment>
-    <comment ref="M28" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 2.7719 %</t>
-      </text>
-    </comment>
-    <comment ref="M35" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.9451 %</t>
-      </text>
-    </comment>
-    <comment ref="M36" authorId="0" shapeId="0">
-      <text>
-        <t>Campaign 1: 1.908 %</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -552,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -887,17 +827,17 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>A1-T1</t>
+          <t>A1-B1</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E9" s="12" t="n"/>
@@ -922,11 +862,11 @@
         <f>IF(AND(ISNUMBER(J9),ISNUMBER(K9)),IF(J9&gt;0,(J9+K9)/J9,""),"")</f>
         <v/>
       </c>
-      <c r="M9" s="13" t="n"/>
-      <c r="N9" s="13" t="n"/>
+      <c r="M9" s="16" t="n"/>
+      <c r="N9" s="16" t="n"/>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P9" s="13" t="n"/>
@@ -939,111 +879,111 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>A1-T2</t>
+          <t>A1-B2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G10" s="16" t="n"/>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G10" s="17" t="n"/>
       <c r="H10" s="3">
         <f>1000-F10</f>
         <v/>
       </c>
-      <c r="I10" s="16" t="n"/>
-      <c r="J10" s="18">
+      <c r="I10" s="17" t="n"/>
+      <c r="J10" s="19">
         <f>IF(AND(ISNUMBER(E10),ISNUMBER(G10)),G10-E10,"")</f>
         <v/>
       </c>
-      <c r="K10" s="18">
+      <c r="K10" s="19">
         <f>IF(AND(ISNUMBER(G10),ISNUMBER(I10)),I10-G10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="19">
+      <c r="L10" s="20">
         <f>IF(AND(ISNUMBER(J10),ISNUMBER(K10)),IF(J10&gt;0,(J10+K10)/J10,""),"")</f>
         <v/>
       </c>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P10" s="17" t="n"/>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>A1-B1</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>A4-B1</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="3">
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="11">
         <f>1000-F11</f>
         <v/>
       </c>
-      <c r="I11" s="16" t="n"/>
-      <c r="J11" s="18">
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="14">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER(G11)),G11-E11,"")</f>
         <v/>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="14">
         <f>IF(AND(ISNUMBER(G11),ISNUMBER(I11)),I11-G11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="19">
+      <c r="L11" s="15">
         <f>IF(AND(ISNUMBER(J11),ISNUMBER(K11)),IF(J11&gt;0,(J11+K11)/J11,""),"")</f>
         <v/>
       </c>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="M11" s="16" t="n"/>
+      <c r="N11" s="16" t="n"/>
+      <c r="O11" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P11" s="17" t="n"/>
+      <c r="P11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>A1-B2</t>
+          <t>A4-B2</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1056,25 +996,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G12" s="16" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G12" s="17" t="n"/>
       <c r="H12" s="3">
         <f>1000-F12</f>
         <v/>
       </c>
-      <c r="I12" s="16" t="n"/>
-      <c r="J12" s="18">
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="19">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER(G12)),G12-E12,"")</f>
         <v/>
       </c>
-      <c r="K12" s="18">
+      <c r="K12" s="19">
         <f>IF(AND(ISNUMBER(G12),ISNUMBER(I12)),I12-G12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="20">
         <f>IF(AND(ISNUMBER(J12),ISNUMBER(K12)),IF(J12&gt;0,(J12+K12)/J12,""),"")</f>
         <v/>
       </c>
@@ -1085,17 +1025,17 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P12" s="17" t="n"/>
+      <c r="P12" s="18" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>A4-T1</t>
+          <t>A5-T1</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -1105,7 +1045,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>organic</t>
+          <t>aqueous</t>
         </is>
       </c>
       <c r="E13" s="12" t="n"/>
@@ -1130,11 +1070,11 @@
         <f>IF(AND(ISNUMBER(J13),ISNUMBER(K13)),IF(J13&gt;0,(J13+K13)/J13,""),"")</f>
         <v/>
       </c>
-      <c r="M13" s="13" t="n"/>
-      <c r="N13" s="13" t="n"/>
+      <c r="M13" s="16" t="n"/>
+      <c r="N13" s="16" t="n"/>
       <c r="O13" s="11" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
+          <t>n/a: by difference</t>
         </is>
       </c>
       <c r="P13" s="13" t="n"/>
@@ -1142,12 +1082,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>A4-T2</t>
+          <t>A5-T2</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1157,101 +1097,101 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G14" s="16" t="n"/>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G14" s="17" t="n"/>
       <c r="H14" s="3">
         <f>1000-F14</f>
         <v/>
       </c>
-      <c r="I14" s="16" t="n"/>
-      <c r="J14" s="18">
+      <c r="I14" s="17" t="n"/>
+      <c r="J14" s="19">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER(G14)),G14-E14,"")</f>
         <v/>
       </c>
-      <c r="K14" s="18">
+      <c r="K14" s="19">
         <f>IF(AND(ISNUMBER(G14),ISNUMBER(I14)),I14-G14,"")</f>
         <v/>
       </c>
-      <c r="L14" s="19">
+      <c r="L14" s="20">
         <f>IF(AND(ISNUMBER(J14),ISNUMBER(K14)),IF(J14&gt;0,(J14+K14)/J14,""),"")</f>
         <v/>
       </c>
-      <c r="M14" s="17" t="n"/>
-      <c r="N14" s="17" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P14" s="17" t="n"/>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P14" s="18" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>A4</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>A4-B1</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>B2-B1</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="3">
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="11">
         <f>1000-F15</f>
         <v/>
       </c>
-      <c r="I15" s="16" t="n"/>
-      <c r="J15" s="18">
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="14">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER(G15)),G15-E15,"")</f>
         <v/>
       </c>
-      <c r="K15" s="18">
+      <c r="K15" s="14">
         <f>IF(AND(ISNUMBER(G15),ISNUMBER(I15)),I15-G15,"")</f>
         <v/>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="15">
         <f>IF(AND(ISNUMBER(J15),ISNUMBER(K15)),IF(J15&gt;0,(J15+K15)/J15,""),"")</f>
         <v/>
       </c>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="M15" s="16" t="n"/>
+      <c r="N15" s="16" t="n"/>
+      <c r="O15" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P15" s="17" t="n"/>
+      <c r="P15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>A4-B2</t>
+          <t>B2-B2</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1264,25 +1204,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G16" s="16" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G16" s="17" t="n"/>
       <c r="H16" s="3">
         <f>1000-F16</f>
         <v/>
       </c>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="18">
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="19">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER(G16)),G16-E16,"")</f>
         <v/>
       </c>
-      <c r="K16" s="18">
+      <c r="K16" s="19">
         <f>IF(AND(ISNUMBER(G16),ISNUMBER(I16)),I16-G16,"")</f>
         <v/>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="20">
         <f>IF(AND(ISNUMBER(J16),ISNUMBER(K16)),IF(J16&gt;0,(J16+K16)/J16,""),"")</f>
         <v/>
       </c>
@@ -1293,22 +1233,22 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P16" s="17" t="n"/>
+      <c r="P16" s="18" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>A5-T1</t>
+          <t>B3-B1</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -1338,8 +1278,8 @@
         <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),IF(J17&gt;0,(J17+K17)/J17,""),"")</f>
         <v/>
       </c>
-      <c r="M17" s="20" t="n"/>
-      <c r="N17" s="20" t="n"/>
+      <c r="M17" s="16" t="n"/>
+      <c r="N17" s="16" t="n"/>
       <c r="O17" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
@@ -1350,17 +1290,17 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>A5-T2</t>
+          <t>B3-B2</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1368,25 +1308,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E18" s="16" t="n"/>
-      <c r="F18" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G18" s="16" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="17" t="n"/>
       <c r="H18" s="3">
         <f>1000-F18</f>
         <v/>
       </c>
-      <c r="I18" s="16" t="n"/>
-      <c r="J18" s="18">
+      <c r="I18" s="17" t="n"/>
+      <c r="J18" s="19">
         <f>IF(AND(ISNUMBER(E18),ISNUMBER(G18)),G18-E18,"")</f>
         <v/>
       </c>
-      <c r="K18" s="18">
+      <c r="K18" s="19">
         <f>IF(AND(ISNUMBER(G18),ISNUMBER(I18)),I18-G18,"")</f>
         <v/>
       </c>
-      <c r="L18" s="19">
+      <c r="L18" s="20">
         <f>IF(AND(ISNUMBER(J18),ISNUMBER(K18)),IF(J18&gt;0,(J18+K18)/J18,""),"")</f>
         <v/>
       </c>
@@ -1397,69 +1337,69 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P18" s="17" t="n"/>
+      <c r="P18" s="18" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>A5-B1</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>B4-B1</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Inferior</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="3">
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="11">
         <f>1000-F19</f>
         <v/>
       </c>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="18">
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="14">
         <f>IF(AND(ISNUMBER(E19),ISNUMBER(G19)),G19-E19,"")</f>
         <v/>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="14">
         <f>IF(AND(ISNUMBER(G19),ISNUMBER(I19)),I19-G19,"")</f>
         <v/>
       </c>
-      <c r="L19" s="19">
+      <c r="L19" s="15">
         <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
         <v/>
       </c>
-      <c r="M19" s="17" t="n"/>
-      <c r="N19" s="17" t="n"/>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P19" s="17" t="n"/>
+      <c r="M19" s="16" t="n"/>
+      <c r="N19" s="16" t="n"/>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>A5-B2</t>
+          <t>B4-B2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1469,49 +1409,49 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G20" s="16" t="n"/>
+          <t>aqueous</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="17" t="n"/>
       <c r="H20" s="3">
         <f>1000-F20</f>
         <v/>
       </c>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="18">
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="19">
         <f>IF(AND(ISNUMBER(E20),ISNUMBER(G20)),G20-E20,"")</f>
         <v/>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="19">
         <f>IF(AND(ISNUMBER(G20),ISNUMBER(I20)),I20-G20,"")</f>
         <v/>
       </c>
-      <c r="L20" s="19">
+      <c r="L20" s="20">
         <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
         <v/>
       </c>
-      <c r="M20" s="17" t="n"/>
-      <c r="N20" s="17" t="n"/>
+      <c r="M20" s="5" t="n"/>
+      <c r="N20" s="5" t="n"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P20" s="17" t="n"/>
+          <t>n/a: by difference</t>
+        </is>
+      </c>
+      <c r="P20" s="18" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>B2-B1</t>
+          <t>F5-B1</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -1546,8 +1486,8 @@
         <f>IF(AND(ISNUMBER(J21),ISNUMBER(K21)),IF(J21&gt;0,(J21+K21)/J21,""),"")</f>
         <v/>
       </c>
-      <c r="M21" s="20" t="n"/>
-      <c r="N21" s="20" t="n"/>
+      <c r="M21" s="16" t="n"/>
+      <c r="N21" s="16" t="n"/>
       <c r="O21" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
@@ -1558,12 +1498,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>B2-B2</t>
+          <t>F5-B2</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1576,25 +1516,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G22" s="16" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G22" s="17" t="n"/>
       <c r="H22" s="3">
         <f>1000-F22</f>
         <v/>
       </c>
-      <c r="I22" s="16" t="n"/>
-      <c r="J22" s="18">
+      <c r="I22" s="17" t="n"/>
+      <c r="J22" s="19">
         <f>IF(AND(ISNUMBER(E22),ISNUMBER(G22)),G22-E22,"")</f>
         <v/>
       </c>
-      <c r="K22" s="18">
+      <c r="K22" s="19">
         <f>IF(AND(ISNUMBER(G22),ISNUMBER(I22)),I22-G22,"")</f>
         <v/>
       </c>
-      <c r="L22" s="19">
+      <c r="L22" s="20">
         <f>IF(AND(ISNUMBER(J22),ISNUMBER(K22)),IF(J22&gt;0,(J22+K22)/J22,""),"")</f>
         <v/>
       </c>
@@ -1605,17 +1545,17 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P22" s="17" t="n"/>
+      <c r="P22" s="18" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>B3-B1</t>
+          <t>BIN6-B1</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -1650,8 +1590,8 @@
         <f>IF(AND(ISNUMBER(J23),ISNUMBER(K23)),IF(J23&gt;0,(J23+K23)/J23,""),"")</f>
         <v/>
       </c>
-      <c r="M23" s="20" t="n"/>
-      <c r="N23" s="20" t="n"/>
+      <c r="M23" s="16" t="n"/>
+      <c r="N23" s="16" t="n"/>
       <c r="O23" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
@@ -1662,12 +1602,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>BIN6</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>B3-B2</t>
+          <t>BIN6-B2</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1680,25 +1620,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G24" s="16" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G24" s="17" t="n"/>
       <c r="H24" s="3">
         <f>1000-F24</f>
         <v/>
       </c>
-      <c r="I24" s="16" t="n"/>
-      <c r="J24" s="18">
+      <c r="I24" s="17" t="n"/>
+      <c r="J24" s="19">
         <f>IF(AND(ISNUMBER(E24),ISNUMBER(G24)),G24-E24,"")</f>
         <v/>
       </c>
-      <c r="K24" s="18">
+      <c r="K24" s="19">
         <f>IF(AND(ISNUMBER(G24),ISNUMBER(I24)),I24-G24,"")</f>
         <v/>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="20">
         <f>IF(AND(ISNUMBER(J24),ISNUMBER(K24)),IF(J24&gt;0,(J24+K24)/J24,""),"")</f>
         <v/>
       </c>
@@ -1709,22 +1649,22 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P24" s="17" t="n"/>
+      <c r="P24" s="18" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>B4-B1</t>
+          <t>I2-T1</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1754,8 +1694,8 @@
         <f>IF(AND(ISNUMBER(J25),ISNUMBER(K25)),IF(J25&gt;0,(J25+K25)/J25,""),"")</f>
         <v/>
       </c>
-      <c r="M25" s="20" t="n"/>
-      <c r="N25" s="20" t="n"/>
+      <c r="M25" s="16" t="n"/>
+      <c r="N25" s="16" t="n"/>
       <c r="O25" s="11" t="inlineStr">
         <is>
           <t>n/a: by difference</t>
@@ -1766,17 +1706,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>B4-B2</t>
+          <t>I2-T2</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1784,25 +1724,25 @@
           <t>aqueous</t>
         </is>
       </c>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G26" s="16" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="G26" s="17" t="n"/>
       <c r="H26" s="3">
         <f>1000-F26</f>
         <v/>
       </c>
-      <c r="I26" s="16" t="n"/>
-      <c r="J26" s="18">
+      <c r="I26" s="17" t="n"/>
+      <c r="J26" s="19">
         <f>IF(AND(ISNUMBER(E26),ISNUMBER(G26)),G26-E26,"")</f>
         <v/>
       </c>
-      <c r="K26" s="18">
+      <c r="K26" s="19">
         <f>IF(AND(ISNUMBER(G26),ISNUMBER(I26)),I26-G26,"")</f>
         <v/>
       </c>
-      <c r="L26" s="19">
+      <c r="L26" s="20">
         <f>IF(AND(ISNUMBER(J26),ISNUMBER(K26)),IF(J26&gt;0,(J26+K26)/J26,""),"")</f>
         <v/>
       </c>
@@ -1813,542 +1753,17 @@
           <t>n/a: by difference</t>
         </is>
       </c>
-      <c r="P26" s="17" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>F5-T1</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="11">
-        <f>1000-F27</f>
-        <v/>
-      </c>
-      <c r="I27" s="12" t="n"/>
-      <c r="J27" s="14">
-        <f>IF(AND(ISNUMBER(E27),ISNUMBER(G27)),G27-E27,"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="14">
-        <f>IF(AND(ISNUMBER(G27),ISNUMBER(I27)),I27-G27,"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="15">
-        <f>IF(AND(ISNUMBER(J27),ISNUMBER(K27)),IF(J27&gt;0,(J27+K27)/J27,""),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="13" t="n"/>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="11" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P27" s="13" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>F5-T2</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="3">
-        <f>1000-F28</f>
-        <v/>
-      </c>
-      <c r="I28" s="16" t="n"/>
-      <c r="J28" s="18">
-        <f>IF(AND(ISNUMBER(E28),ISNUMBER(G28)),G28-E28,"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="18">
-        <f>IF(AND(ISNUMBER(G28),ISNUMBER(I28)),I28-G28,"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="19">
-        <f>IF(AND(ISNUMBER(J28),ISNUMBER(K28)),IF(J28&gt;0,(J28+K28)/J28,""),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="17" t="n"/>
-      <c r="N28" s="17" t="n"/>
-      <c r="O28" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P28" s="17" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>F5-B1</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="3">
-        <f>1000-F29</f>
-        <v/>
-      </c>
-      <c r="I29" s="16" t="n"/>
-      <c r="J29" s="18">
-        <f>IF(AND(ISNUMBER(E29),ISNUMBER(G29)),G29-E29,"")</f>
-        <v/>
-      </c>
-      <c r="K29" s="18">
-        <f>IF(AND(ISNUMBER(G29),ISNUMBER(I29)),I29-G29,"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="19">
-        <f>IF(AND(ISNUMBER(J29),ISNUMBER(K29)),IF(J29&gt;0,(J29+K29)/J29,""),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="5" t="n"/>
-      <c r="N29" s="5" t="n"/>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P29" s="17" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>F5</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>F5-B2</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="3">
-        <f>1000-F30</f>
-        <v/>
-      </c>
-      <c r="I30" s="16" t="n"/>
-      <c r="J30" s="18">
-        <f>IF(AND(ISNUMBER(E30),ISNUMBER(G30)),G30-E30,"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="18">
-        <f>IF(AND(ISNUMBER(G30),ISNUMBER(I30)),I30-G30,"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="19">
-        <f>IF(AND(ISNUMBER(J30),ISNUMBER(K30)),IF(J30&gt;0,(J30+K30)/J30,""),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="5" t="n"/>
-      <c r="N30" s="5" t="n"/>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P30" s="17" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>BIN6</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>BIN6-B1</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="n"/>
-      <c r="F31" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="11">
-        <f>1000-F31</f>
-        <v/>
-      </c>
-      <c r="I31" s="12" t="n"/>
-      <c r="J31" s="14">
-        <f>IF(AND(ISNUMBER(E31),ISNUMBER(G31)),G31-E31,"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="14">
-        <f>IF(AND(ISNUMBER(G31),ISNUMBER(I31)),I31-G31,"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="15">
-        <f>IF(AND(ISNUMBER(J31),ISNUMBER(K31)),IF(J31&gt;0,(J31+K31)/J31,""),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="20" t="n"/>
-      <c r="N31" s="20" t="n"/>
-      <c r="O31" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P31" s="13" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>BIN6</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>BIN6-B2</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="3">
-        <f>1000-F32</f>
-        <v/>
-      </c>
-      <c r="I32" s="16" t="n"/>
-      <c r="J32" s="18">
-        <f>IF(AND(ISNUMBER(E32),ISNUMBER(G32)),G32-E32,"")</f>
-        <v/>
-      </c>
-      <c r="K32" s="18">
-        <f>IF(AND(ISNUMBER(G32),ISNUMBER(I32)),I32-G32,"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="19">
-        <f>IF(AND(ISNUMBER(J32),ISNUMBER(K32)),IF(J32&gt;0,(J32+K32)/J32,""),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="5" t="n"/>
-      <c r="N32" s="5" t="n"/>
-      <c r="O32" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P32" s="17" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>I2-T1</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="n"/>
-      <c r="F33" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G33" s="12" t="n"/>
-      <c r="H33" s="11">
-        <f>1000-F33</f>
-        <v/>
-      </c>
-      <c r="I33" s="12" t="n"/>
-      <c r="J33" s="14">
-        <f>IF(AND(ISNUMBER(E33),ISNUMBER(G33)),G33-E33,"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="14">
-        <f>IF(AND(ISNUMBER(G33),ISNUMBER(I33)),I33-G33,"")</f>
-        <v/>
-      </c>
-      <c r="L33" s="15">
-        <f>IF(AND(ISNUMBER(J33),ISNUMBER(K33)),IF(J33&gt;0,(J33+K33)/J33,""),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="20" t="n"/>
-      <c r="N33" s="20" t="n"/>
-      <c r="O33" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P33" s="13" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>I2-T2</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="3">
-        <f>1000-F34</f>
-        <v/>
-      </c>
-      <c r="I34" s="16" t="n"/>
-      <c r="J34" s="18">
-        <f>IF(AND(ISNUMBER(E34),ISNUMBER(G34)),G34-E34,"")</f>
-        <v/>
-      </c>
-      <c r="K34" s="18">
-        <f>IF(AND(ISNUMBER(G34),ISNUMBER(I34)),I34-G34,"")</f>
-        <v/>
-      </c>
-      <c r="L34" s="19">
-        <f>IF(AND(ISNUMBER(J34),ISNUMBER(K34)),IF(J34&gt;0,(J34+K34)/J34,""),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="5" t="n"/>
-      <c r="N34" s="5" t="n"/>
-      <c r="O34" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P34" s="17" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>I2-B1</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="3">
-        <f>1000-F35</f>
-        <v/>
-      </c>
-      <c r="I35" s="16" t="n"/>
-      <c r="J35" s="18">
-        <f>IF(AND(ISNUMBER(E35),ISNUMBER(G35)),G35-E35,"")</f>
-        <v/>
-      </c>
-      <c r="K35" s="18">
-        <f>IF(AND(ISNUMBER(G35),ISNUMBER(I35)),I35-G35,"")</f>
-        <v/>
-      </c>
-      <c r="L35" s="19">
-        <f>IF(AND(ISNUMBER(J35),ISNUMBER(K35)),IF(J35&gt;0,(J35+K35)/J35,""),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="17" t="n"/>
-      <c r="N35" s="17" t="n"/>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P35" s="17" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>I2-B2</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Inferior</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>organic</t>
-        </is>
-      </c>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="3">
-        <f>1000-F36</f>
-        <v/>
-      </c>
-      <c r="I36" s="16" t="n"/>
-      <c r="J36" s="18">
-        <f>IF(AND(ISNUMBER(E36),ISNUMBER(G36)),G36-E36,"")</f>
-        <v/>
-      </c>
-      <c r="K36" s="18">
-        <f>IF(AND(ISNUMBER(G36),ISNUMBER(I36)),I36-G36,"")</f>
-        <v/>
-      </c>
-      <c r="L36" s="19">
-        <f>IF(AND(ISNUMBER(J36),ISNUMBER(K36)),IF(J36&gt;0,(J36+K36)/J36,""),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="17" t="n"/>
-      <c r="N36" s="17" t="n"/>
-      <c r="O36" s="3" t="inlineStr">
-        <is>
-          <t>fresh: type the new KF</t>
-        </is>
-      </c>
-      <c r="P36" s="17" t="n"/>
+      <c r="P26" s="18" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <dataValidations count="2">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 E27:G27 E28:G28 E29:G29 E30:G30 E31:G31 E32:G32 E33:G33 E34:G34 E35:G35 E36:G36 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
-      <formula1>0</formula1>
-      <formula2>100</formula2>
-    </dataValidation>
-    <dataValidation sqref="M9:N9 M10:N10 M13:N13 M14:N14 M19:N19 M20:N20 M27:N27 M28:N28 M35:N35 M36:N36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+  <dataValidations count="1">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 E21:G21 E22:G22 E23:G23 E24:G24 E25:G25 E26:G26 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>